<commit_message>
Cleaned Code, but no note
</commit_message>
<xml_diff>
--- a/blank_form.xlsx
+++ b/blank_form.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\Form Maker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29E15DC1-9F64-4BA2-8680-9C708479F677}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B01568B0-C2B5-4D5B-8A51-239AC8109DF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{13A5ADAB-B568-4D4E-B2A7-A9C799E1CA91}"/>
   </bookViews>
@@ -23021,8 +23021,7 @@
       <c r="G48" s="14"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A43:G48"/>
+  <mergeCells count="8">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A3:G3"/>

</xml_diff>

<commit_message>
Update blank form, fix selection update bug
</commit_message>
<xml_diff>
--- a/blank_form.xlsx
+++ b/blank_form.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\Form Maker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B01568B0-C2B5-4D5B-8A51-239AC8109DF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36E5E193-92F8-4EBB-94DE-E5F7BB9CD73C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{13A5ADAB-B568-4D4E-B2A7-A9C799E1CA91}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t xml:space="preserve">明泰冷氣有限公司 </t>
   </si>
@@ -84,11 +84,6 @@
   </si>
   <si>
     <t>小計</t>
-  </si>
-  <si>
-    <t>1.本估價單30天內有效.如經同意施作.請簽名回傳
-2.估價單施工時間為正常上班日(星期一至五，上午九點至下午五點。），如需特殊時段施工，需另行報價。</t>
-    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>營業稅</t>
@@ -22257,6 +22252,61 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>247649</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1924050</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="圖片 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{67AA03C3-33D3-4C74-B08A-17A17DE5B4E2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="10753724"/>
+          <a:ext cx="2266950" cy="1790701"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 佈景主題">
   <a:themeElements>
@@ -22948,7 +22998,7 @@
     </row>
     <row r="41" spans="1:7" s="9" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
       <c r="E41" s="9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="12"/>
@@ -22959,15 +23009,13 @@
       <c r="C42" s="9"/>
       <c r="D42" s="9"/>
       <c r="E42" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="8"/>
     </row>
     <row r="43" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="13" t="s">
-        <v>12</v>
-      </c>
+      <c r="A43" s="13"/>
       <c r="B43" s="13"/>
       <c r="C43" s="13"/>
       <c r="D43" s="13"/>
@@ -23022,17 +23070,18 @@
     </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C7:D7"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A3:G3"/>
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="C7:D7"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
revise ui, fix blank_form.xlsx stamp image
</commit_message>
<xml_diff>
--- a/blank_form.xlsx
+++ b/blank_form.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\Form Maker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36E5E193-92F8-4EBB-94DE-E5F7BB9CD73C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBCACF53-840A-48D3-82AB-DD64054F35ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{13A5ADAB-B568-4D4E-B2A7-A9C799E1CA91}"/>
   </bookViews>
@@ -16739,6 +16739,15 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="176" fontId="7" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -16746,15 +16755,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="7" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -22258,14 +22258,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>41</xdr:row>
-      <xdr:rowOff>247649</xdr:rowOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>76199</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>1924050</xdr:colOff>
-      <xdr:row>50</xdr:row>
-      <xdr:rowOff>114300</xdr:rowOff>
+      <xdr:colOff>1524000</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>84044</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -22294,8 +22294,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="10753724"/>
-          <a:ext cx="2266950" cy="1790701"/>
+          <a:off x="0" y="10829924"/>
+          <a:ext cx="1866900" cy="1474695"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -22615,59 +22615,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
     </row>
     <row r="2" spans="1:7" ht="21" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
     </row>
     <row r="3" spans="1:7" ht="21" x14ac:dyDescent="0.25">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="16"/>
+      <c r="B3" s="19"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
     </row>
     <row r="4" spans="1:7" ht="21" x14ac:dyDescent="0.25">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="16"/>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="16"/>
-      <c r="G4" s="16"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="19"/>
     </row>
     <row r="5" spans="1:7" ht="32.25" x14ac:dyDescent="0.25">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="17"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="20"/>
     </row>
     <row r="6" spans="1:7" ht="19.5" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
@@ -22677,20 +22677,20 @@
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
       <c r="E6" s="1"/>
-      <c r="F6" s="18">
+      <c r="F6" s="15">
         <v>45915</v>
       </c>
-      <c r="G6" s="18"/>
+      <c r="G6" s="15"/>
     </row>
     <row r="7" spans="1:7" ht="19.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="20"/>
-      <c r="C7" s="19" t="s">
+      <c r="B7" s="17"/>
+      <c r="C7" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="20"/>
+      <c r="D7" s="17"/>
       <c r="E7" s="5" t="s">
         <v>8</v>
       </c>

</xml_diff>

<commit_message>
fix stamp image size, kill some print function
</commit_message>
<xml_diff>
--- a/blank_form.xlsx
+++ b/blank_form.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\Form Maker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBCACF53-840A-48D3-82AB-DD64054F35ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C40D6233-9F39-4D15-8469-CFF7B305723B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{13A5ADAB-B568-4D4E-B2A7-A9C799E1CA91}"/>
   </bookViews>
@@ -22263,9 +22263,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>1524000</xdr:colOff>
-      <xdr:row>49</xdr:row>
-      <xdr:rowOff>84044</xdr:rowOff>
+      <xdr:colOff>1211580</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>167639</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -22295,7 +22295,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="10829924"/>
-          <a:ext cx="1866900" cy="1474695"/>
+          <a:ext cx="1554480" cy="1348740"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>

<commit_message>
rename item_json file, fix 小計 營業稅 總計, auto 注意事項(送風機 水冷
</commit_message>
<xml_diff>
--- a/blank_form.xlsx
+++ b/blank_form.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\Form Maker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C40D6233-9F39-4D15-8469-CFF7B305723B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{942BC5CD-B119-4628-8D23-8D4B86C3BA6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{13A5ADAB-B568-4D4E-B2A7-A9C799E1CA91}"/>
   </bookViews>
@@ -16693,7 +16693,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -16756,6 +16756,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="5479">
@@ -22258,14 +22261,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>42</xdr:row>
+      <xdr:row>61</xdr:row>
       <xdr:rowOff>76199</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>1211580</xdr:colOff>
-      <xdr:row>48</xdr:row>
-      <xdr:rowOff>167639</xdr:rowOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>186689</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -22604,7 +22607,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15390A6D-3125-435E-A706-0756C42C8156}">
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G67"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.5" customWidth="1"/>
@@ -22981,92 +22984,271 @@
       <c r="G38" s="11"/>
     </row>
     <row r="39" spans="1:7" ht="19.5" x14ac:dyDescent="0.25">
-      <c r="A39" s="5"/>
-      <c r="B39" s="3"/>
-      <c r="C39" s="5"/>
-      <c r="D39" s="5"/>
+      <c r="A39" s="11"/>
+      <c r="B39" s="10"/>
+      <c r="C39" s="11"/>
+      <c r="D39" s="11"/>
       <c r="E39" s="2"/>
       <c r="F39" s="2"/>
-      <c r="G39" s="5"/>
+      <c r="G39" s="11"/>
     </row>
     <row r="40" spans="1:7" s="9" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
-      <c r="E40" s="9" t="s">
+      <c r="A40" s="11"/>
+      <c r="B40" s="10"/>
+      <c r="C40" s="11"/>
+      <c r="D40" s="11"/>
+      <c r="E40" s="2"/>
+      <c r="F40" s="2"/>
+      <c r="G40" s="11"/>
+    </row>
+    <row r="41" spans="1:7" s="9" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="A41" s="11"/>
+      <c r="B41" s="10"/>
+      <c r="C41" s="11"/>
+      <c r="D41" s="11"/>
+      <c r="E41" s="2"/>
+      <c r="F41" s="2"/>
+      <c r="G41" s="11"/>
+    </row>
+    <row r="42" spans="1:7" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="A42" s="11"/>
+      <c r="B42" s="10"/>
+      <c r="C42" s="11"/>
+      <c r="D42" s="11"/>
+      <c r="E42" s="2"/>
+      <c r="F42" s="2"/>
+      <c r="G42" s="11"/>
+    </row>
+    <row r="43" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="11"/>
+      <c r="B43" s="10"/>
+      <c r="C43" s="11"/>
+      <c r="D43" s="11"/>
+      <c r="E43" s="2"/>
+      <c r="F43" s="2"/>
+      <c r="G43" s="11"/>
+    </row>
+    <row r="44" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="11"/>
+      <c r="B44" s="10"/>
+      <c r="C44" s="11"/>
+      <c r="D44" s="11"/>
+      <c r="E44" s="2"/>
+      <c r="F44" s="2"/>
+      <c r="G44" s="11"/>
+    </row>
+    <row r="45" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="11"/>
+      <c r="B45" s="10"/>
+      <c r="C45" s="11"/>
+      <c r="D45" s="11"/>
+      <c r="E45" s="2"/>
+      <c r="F45" s="2"/>
+      <c r="G45" s="11"/>
+    </row>
+    <row r="46" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="11"/>
+      <c r="B46" s="10"/>
+      <c r="C46" s="11"/>
+      <c r="D46" s="11"/>
+      <c r="E46" s="2"/>
+      <c r="F46" s="2"/>
+      <c r="G46" s="11"/>
+    </row>
+    <row r="47" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="11"/>
+      <c r="B47" s="10"/>
+      <c r="C47" s="11"/>
+      <c r="D47" s="11"/>
+      <c r="E47" s="2"/>
+      <c r="F47" s="2"/>
+      <c r="G47" s="11"/>
+    </row>
+    <row r="48" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="11"/>
+      <c r="B48" s="10"/>
+      <c r="C48" s="11"/>
+      <c r="D48" s="11"/>
+      <c r="E48" s="2"/>
+      <c r="F48" s="2"/>
+      <c r="G48" s="11"/>
+    </row>
+    <row r="49" spans="1:7" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="A49" s="11"/>
+      <c r="B49" s="10"/>
+      <c r="C49" s="11"/>
+      <c r="D49" s="11"/>
+      <c r="E49" s="2"/>
+      <c r="F49" s="2"/>
+      <c r="G49" s="11"/>
+    </row>
+    <row r="50" spans="1:7" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="A50" s="11"/>
+      <c r="B50" s="10"/>
+      <c r="C50" s="11"/>
+      <c r="D50" s="11"/>
+      <c r="E50" s="2"/>
+      <c r="F50" s="2"/>
+      <c r="G50" s="11"/>
+    </row>
+    <row r="51" spans="1:7" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="A51" s="11"/>
+      <c r="B51" s="10"/>
+      <c r="C51" s="11"/>
+      <c r="D51" s="11"/>
+      <c r="E51" s="2"/>
+      <c r="F51" s="2"/>
+      <c r="G51" s="11"/>
+    </row>
+    <row r="52" spans="1:7" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="A52" s="11"/>
+      <c r="B52" s="10"/>
+      <c r="C52" s="11"/>
+      <c r="D52" s="11"/>
+      <c r="E52" s="2"/>
+      <c r="F52" s="2"/>
+      <c r="G52" s="11"/>
+    </row>
+    <row r="53" spans="1:7" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="A53" s="11"/>
+      <c r="B53" s="10"/>
+      <c r="C53" s="11"/>
+      <c r="D53" s="11"/>
+      <c r="E53" s="2"/>
+      <c r="F53" s="2"/>
+      <c r="G53" s="11"/>
+    </row>
+    <row r="54" spans="1:7" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="A54" s="11"/>
+      <c r="B54" s="10"/>
+      <c r="C54" s="11"/>
+      <c r="D54" s="11"/>
+      <c r="E54" s="2"/>
+      <c r="F54" s="2"/>
+      <c r="G54" s="11"/>
+    </row>
+    <row r="55" spans="1:7" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="A55" s="11"/>
+      <c r="B55" s="10"/>
+      <c r="C55" s="11"/>
+      <c r="D55" s="11"/>
+      <c r="E55" s="2"/>
+      <c r="F55" s="2"/>
+      <c r="G55" s="11"/>
+    </row>
+    <row r="56" spans="1:7" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="A56" s="11"/>
+      <c r="B56" s="10"/>
+      <c r="C56" s="11"/>
+      <c r="D56" s="11"/>
+      <c r="E56" s="2"/>
+      <c r="F56" s="2"/>
+      <c r="G56" s="11"/>
+    </row>
+    <row r="57" spans="1:7" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="A57" s="11"/>
+      <c r="B57" s="10"/>
+      <c r="C57" s="11"/>
+      <c r="D57" s="11"/>
+      <c r="E57" s="2"/>
+      <c r="F57" s="2"/>
+      <c r="G57" s="11"/>
+    </row>
+    <row r="58" spans="1:7" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="A58" s="5"/>
+      <c r="B58" s="3"/>
+      <c r="C58" s="5"/>
+      <c r="D58" s="5"/>
+      <c r="E58" s="2"/>
+      <c r="F58" s="2"/>
+      <c r="G58" s="5"/>
+    </row>
+    <row r="59" spans="1:7" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="A59" s="9"/>
+      <c r="B59" s="9"/>
+      <c r="C59" s="9"/>
+      <c r="D59" s="9"/>
+      <c r="E59" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="F40" s="4"/>
-      <c r="G40" s="12"/>
+      <c r="F59" s="4"/>
+      <c r="G59" s="12"/>
     </row>
-    <row r="41" spans="1:7" s="9" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
-      <c r="E41" s="9" t="s">
+    <row r="60" spans="1:7" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="A60" s="9"/>
+      <c r="B60" s="9"/>
+      <c r="C60" s="9"/>
+      <c r="D60" s="9"/>
+      <c r="E60" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="F41" s="4"/>
-      <c r="G41" s="12"/>
+      <c r="F60" s="4"/>
+      <c r="G60" s="12"/>
     </row>
-    <row r="42" spans="1:7" ht="19.5" x14ac:dyDescent="0.25">
-      <c r="A42" s="9"/>
-      <c r="B42" s="9"/>
-      <c r="C42" s="9"/>
-      <c r="D42" s="9"/>
-      <c r="E42" s="9" t="s">
+    <row r="61" spans="1:7" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="A61" s="9"/>
+      <c r="B61" s="9"/>
+      <c r="C61" s="9"/>
+      <c r="D61" s="9"/>
+      <c r="E61" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="F42" s="4"/>
-      <c r="G42" s="8"/>
+      <c r="F61" s="4"/>
+      <c r="G61" s="8"/>
     </row>
-    <row r="43" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="13"/>
-      <c r="B43" s="13"/>
-      <c r="C43" s="13"/>
-      <c r="D43" s="13"/>
-      <c r="E43" s="13"/>
-      <c r="F43" s="13"/>
-      <c r="G43" s="13"/>
+    <row r="62" spans="1:7" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="A62" s="13"/>
+      <c r="B62" s="13"/>
+      <c r="C62" s="13"/>
+      <c r="D62" s="13"/>
+      <c r="E62" s="13"/>
+      <c r="F62" s="13"/>
+      <c r="G62" s="13"/>
     </row>
-    <row r="44" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="14"/>
-      <c r="B44" s="14"/>
-      <c r="C44" s="14"/>
-      <c r="D44" s="14"/>
-      <c r="E44" s="14"/>
-      <c r="F44" s="14"/>
-      <c r="G44" s="14"/>
+    <row r="63" spans="1:7" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="A63" s="14"/>
+      <c r="B63" s="14"/>
+      <c r="C63" s="14"/>
+      <c r="D63" s="14"/>
+      <c r="E63" s="14"/>
+      <c r="F63" s="14"/>
+      <c r="G63" s="14"/>
     </row>
-    <row r="45" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="14"/>
-      <c r="B45" s="14"/>
-      <c r="C45" s="14"/>
-      <c r="D45" s="14"/>
-      <c r="E45" s="14"/>
-      <c r="F45" s="14"/>
-      <c r="G45" s="14"/>
+    <row r="64" spans="1:7" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="A64" s="14"/>
+      <c r="B64" s="14"/>
+      <c r="C64" s="14"/>
+      <c r="D64" s="14"/>
+      <c r="E64" s="14"/>
+      <c r="F64" s="14"/>
+      <c r="G64" s="14"/>
     </row>
-    <row r="46" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="14"/>
-      <c r="B46" s="14"/>
-      <c r="C46" s="14"/>
-      <c r="D46" s="14"/>
-      <c r="E46" s="14"/>
-      <c r="F46" s="14"/>
-      <c r="G46" s="14"/>
+    <row r="65" spans="1:7" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="A65" s="14"/>
+      <c r="B65" s="14"/>
+      <c r="C65" s="14"/>
+      <c r="D65" s="14"/>
+      <c r="E65" s="14"/>
+      <c r="F65" s="14"/>
+      <c r="G65" s="14"/>
     </row>
-    <row r="47" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="14"/>
-      <c r="B47" s="14"/>
-      <c r="C47" s="14"/>
-      <c r="D47" s="14"/>
-      <c r="E47" s="14"/>
-      <c r="F47" s="14"/>
-      <c r="G47" s="14"/>
+    <row r="66" spans="1:7" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="A66" s="14"/>
+      <c r="B66" s="14"/>
+      <c r="C66" s="14"/>
+      <c r="D66" s="14"/>
+      <c r="E66" s="14"/>
+      <c r="F66" s="14"/>
+      <c r="G66" s="14"/>
     </row>
-    <row r="48" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="14"/>
-      <c r="B48" s="14"/>
-      <c r="C48" s="14"/>
-      <c r="D48" s="14"/>
-      <c r="E48" s="14"/>
-      <c r="F48" s="14"/>
-      <c r="G48" s="14"/>
+    <row r="67" spans="1:7" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="A67" s="14"/>
+      <c r="B67" s="14"/>
+      <c r="C67" s="14"/>
+      <c r="D67" s="14"/>
+      <c r="E67" s="14"/>
+      <c r="F67" s="14"/>
+      <c r="G67" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>

<commit_message>
adjust stamp image, add formula export
</commit_message>
<xml_diff>
--- a/blank_form.xlsx
+++ b/blank_form.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\Form Maker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{942BC5CD-B119-4628-8D23-8D4B86C3BA6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64109742-820D-49B7-A1C0-D19C6A53507D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{13A5ADAB-B568-4D4E-B2A7-A9C799E1CA91}"/>
   </bookViews>
@@ -16739,6 +16739,9 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="176" fontId="7" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -16756,9 +16759,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="5479">
@@ -22259,16 +22259,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3019426</xdr:colOff>
       <xdr:row>61</xdr:row>
-      <xdr:rowOff>76199</xdr:rowOff>
+      <xdr:rowOff>9525</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>1211580</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>177928</xdr:colOff>
       <xdr:row>66</xdr:row>
-      <xdr:rowOff>186689</xdr:rowOff>
+      <xdr:rowOff>93040</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -22297,8 +22297,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="10829924"/>
-          <a:ext cx="1554480" cy="1348740"/>
+          <a:off x="3362326" y="15240000"/>
+          <a:ext cx="1787652" cy="1321765"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -22618,59 +22618,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
     </row>
     <row r="2" spans="1:7" ht="21" x14ac:dyDescent="0.25">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
     </row>
     <row r="3" spans="1:7" ht="21" x14ac:dyDescent="0.25">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="19"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
+      <c r="G3" s="20"/>
     </row>
     <row r="4" spans="1:7" ht="21" x14ac:dyDescent="0.25">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="19"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="20"/>
     </row>
     <row r="5" spans="1:7" ht="32.25" x14ac:dyDescent="0.25">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="20"/>
-      <c r="C5" s="20"/>
-      <c r="D5" s="20"/>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="20"/>
+      <c r="B5" s="21"/>
+      <c r="C5" s="21"/>
+      <c r="D5" s="21"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="21"/>
     </row>
     <row r="6" spans="1:7" ht="19.5" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
@@ -22680,20 +22680,20 @@
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
       <c r="E6" s="1"/>
-      <c r="F6" s="15">
+      <c r="F6" s="16">
         <v>45915</v>
       </c>
-      <c r="G6" s="15"/>
+      <c r="G6" s="16"/>
     </row>
     <row r="7" spans="1:7" ht="19.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="16" t="s">
+      <c r="A7" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="17"/>
-      <c r="C7" s="16" t="s">
+      <c r="B7" s="18"/>
+      <c r="C7" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="17"/>
+      <c r="D7" s="18"/>
       <c r="E7" s="5" t="s">
         <v>8</v>
       </c>
@@ -23168,7 +23168,7 @@
       <c r="B59" s="9"/>
       <c r="C59" s="9"/>
       <c r="D59" s="9"/>
-      <c r="E59" s="21" t="s">
+      <c r="E59" s="15" t="s">
         <v>11</v>
       </c>
       <c r="F59" s="4"/>
@@ -23179,7 +23179,7 @@
       <c r="B60" s="9"/>
       <c r="C60" s="9"/>
       <c r="D60" s="9"/>
-      <c r="E60" s="21" t="s">
+      <c r="E60" s="15" t="s">
         <v>12</v>
       </c>
       <c r="F60" s="4"/>
@@ -23190,7 +23190,7 @@
       <c r="B61" s="9"/>
       <c r="C61" s="9"/>
       <c r="D61" s="9"/>
-      <c r="E61" s="21" t="s">
+      <c r="E61" s="15" t="s">
         <v>13</v>
       </c>
       <c r="F61" s="4"/>

</xml_diff>